<commit_message>
Substitui bases de meta e vendas para acompanhamento do evento de amanha
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/meta_supervisor.xlsx
+++ b/data/meta_supervisor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christian.roque\Desktop\Total_Day\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{943C93E3-D57A-4BC5-ABA6-C04BD224D8F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5496804-AEA2-4401-A746-E46D27939337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha2" sheetId="3" r:id="rId1"/>
@@ -36,13 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
-  <si>
-    <t>PI</t>
-  </si>
-  <si>
-    <t>MA</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>cod_filial</t>
   </si>
@@ -56,42 +50,6 @@
     <t>meta supervisão</t>
   </si>
   <si>
-    <t>FERNANDO NOBRE MARTINS</t>
-  </si>
-  <si>
-    <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
-  </si>
-  <si>
-    <t>JOSE MARIA FERNANDES FONTENELE</t>
-  </si>
-  <si>
-    <t>MARIA ECILIA ALVES DOS SANTOS</t>
-  </si>
-  <si>
-    <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
-  </si>
-  <si>
-    <t>FERNANDA DA SILVA OLIVEIRA</t>
-  </si>
-  <si>
-    <t>JOSE FLAVIO DE SA AZEVEDO</t>
-  </si>
-  <si>
-    <t>SALDANHA JUNIOR</t>
-  </si>
-  <si>
-    <t>PAULO CESAR DAMACENA LEMOS - HB</t>
-  </si>
-  <si>
-    <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
-  </si>
-  <si>
-    <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
-  </si>
-  <si>
-    <t>JONATHAS SANTOS ANDRADE - FARMA</t>
-  </si>
-  <si>
     <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
   </si>
   <si>
@@ -101,19 +59,7 @@
     <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
   </si>
   <si>
-    <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
-  </si>
-  <si>
-    <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
-  </si>
-  <si>
-    <t>BERNARDO TEIXEIRA COSTA NETO</t>
-  </si>
-  <si>
-    <t>RILARY DIENIFER TRAUTMANN LIMA</t>
-  </si>
-  <si>
-    <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+    <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
   </si>
 </sst>
 </file>
@@ -121,7 +67,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -152,7 +98,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -487,7 +433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A56F8248-F6E2-4ACE-AE7B-74CB24EA34E5}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.5" bestFit="1" customWidth="1"/>
@@ -497,296 +443,72 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B2">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="1">
-        <v>1269728.7716268308</v>
+        <v>380861.4572787378</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B3">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D3" s="1">
-        <v>545748.29481634218</v>
+        <v>622707.10011262679</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B4">
-        <v>106</v>
+        <v>146</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D4" s="1">
-        <v>530239.16272349597</v>
+        <v>679666.25696659449</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B5">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D5" s="1">
-        <v>558770.79818590835</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6">
-        <v>46</v>
-      </c>
-      <c r="C6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="1">
-        <v>453598.2330648721</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>3</v>
-      </c>
-      <c r="B7">
-        <v>43</v>
-      </c>
-      <c r="C7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="1">
-        <v>401184.36881949956</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>3</v>
-      </c>
-      <c r="B8">
-        <v>132</v>
-      </c>
-      <c r="C8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="1">
-        <v>379527.96466602071</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>3</v>
-      </c>
-      <c r="B9">
-        <v>2</v>
-      </c>
-      <c r="C9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="1">
-        <v>302203.85443036543</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>7</v>
-      </c>
-      <c r="B10">
-        <v>98</v>
-      </c>
-      <c r="C10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" s="1">
-        <v>806098.12525992142</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>7</v>
-      </c>
-      <c r="B11">
-        <v>100</v>
-      </c>
-      <c r="C11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D11" s="1">
-        <v>425730.7363007958</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>7</v>
-      </c>
-      <c r="B12">
-        <v>95</v>
-      </c>
-      <c r="C12" t="s">
-        <v>16</v>
-      </c>
-      <c r="D12" s="1">
-        <v>230789.9599278653</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>7</v>
-      </c>
-      <c r="B13">
-        <v>50</v>
-      </c>
-      <c r="C13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="1">
-        <v>194216.32184475061</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>9</v>
-      </c>
-      <c r="B14">
-        <v>146</v>
-      </c>
-      <c r="C14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="1">
-        <v>429705.98547714611</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>9</v>
-      </c>
-      <c r="B15">
-        <v>135</v>
-      </c>
-      <c r="C15" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="1">
-        <v>374775.32536699361</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>9</v>
-      </c>
-      <c r="B16">
-        <v>147</v>
-      </c>
-      <c r="C16" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" s="1">
-        <v>364830.59568110958</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>0</v>
-      </c>
-      <c r="B17">
-        <v>39</v>
-      </c>
-      <c r="C17" t="s">
-        <v>21</v>
-      </c>
-      <c r="D17" s="1">
-        <v>967286.30113893328</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B18">
-        <v>69</v>
-      </c>
-      <c r="C18" t="s">
-        <v>22</v>
-      </c>
-      <c r="D18" s="1">
-        <v>691106.01136106486</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>1</v>
-      </c>
-      <c r="B19">
-        <v>38</v>
-      </c>
-      <c r="C19" t="s">
-        <v>23</v>
-      </c>
-      <c r="D19" s="1">
-        <v>645011.17730252154</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>1</v>
-      </c>
-      <c r="B20">
-        <v>114</v>
-      </c>
-      <c r="C20" t="s">
-        <v>24</v>
-      </c>
-      <c r="D20" s="1">
-        <v>519393.11883568548</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>1</v>
-      </c>
-      <c r="B21">
-        <v>120</v>
-      </c>
-      <c r="C21" t="s">
-        <v>25</v>
-      </c>
-      <c r="D21" s="1">
-        <v>474510.38562012545</v>
+        <v>116765.18564204073</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adiciona aba de Gerentes e atualiza bases do evento
Apuracao por gerente soma o pedido pelo codigo em todas as filiais e usa a
filial do cadastro de meta para o filtro; pedidos de gerentes sem meta
aparecem em nota. Inclui meta_gerente.xlsx, nova meta de supervisores,
vendas com COD_GERENTE e remove meta_rca.xlsx, que nao e mais usada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/meta_supervisor.xlsx
+++ b/data/meta_supervisor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christian.roque\Desktop\Total_Day\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5496804-AEA2-4401-A746-E46D27939337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{206B6471-A82B-4100-A8EB-6CCA77C26D38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>cod_filial</t>
   </si>
@@ -56,10 +56,61 @@
     <t>JOSE CAETANO DA SILVA JUNIOR</t>
   </si>
   <si>
-    <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
-  </si>
-  <si>
-    <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+    <t>FERNANDO NOBRE MARTINS</t>
+  </si>
+  <si>
+    <t>JOSE MARIA FERNANDES FONTENELE</t>
+  </si>
+  <si>
+    <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+  </si>
+  <si>
+    <t>PI</t>
+  </si>
+  <si>
+    <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+  </si>
+  <si>
+    <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+  </si>
+  <si>
+    <t>FERNANDA DA SILVA OLIVEIRA</t>
+  </si>
+  <si>
+    <t>JOSE FLAVIO DE SA AZEVEDO</t>
+  </si>
+  <si>
+    <t>SALDANHA JUNIOR</t>
+  </si>
+  <si>
+    <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+  </si>
+  <si>
+    <t>MA</t>
+  </si>
+  <si>
+    <t>BERNARDO TEIXEIRA COSTA NETO</t>
+  </si>
+  <si>
+    <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+  </si>
+  <si>
+    <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+  </si>
+  <si>
+    <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+  </si>
+  <si>
+    <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+  </si>
+  <si>
+    <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+  </si>
+  <si>
+    <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+  </si>
+  <si>
+    <t>SUPERVISOR FARMA - PE</t>
   </si>
 </sst>
 </file>
@@ -433,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A56F8248-F6E2-4ACE-AE7B-74CB24EA34E5}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.5" bestFit="1" customWidth="1"/>
@@ -457,58 +508,268 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B2">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="1">
-        <v>380861.4572787378</v>
+        <v>2076618.5327999997</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B3">
-        <v>135</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D3" s="1">
-        <v>622707.10011262679</v>
+        <v>1124835.0385999999</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>145</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1124835.0385999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B4">
+      <c r="B5">
+        <v>69</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="1">
+        <v>686508.20389668294</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="1">
+        <v>975390.78610331658</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="1">
+        <v>1746892.3292411075</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>3</v>
+      </c>
+      <c r="B8">
+        <v>132</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1061194.1935783071</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="1">
+        <v>896554.42641040857</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>46</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1231506.3807701776</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
+        <v>38</v>
+      </c>
+      <c r="C11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="1">
+        <v>727113.31019710645</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12">
+        <v>120</v>
+      </c>
+      <c r="C12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="1">
+        <v>402229.44315466011</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13">
+        <v>114</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="1">
+        <v>480568.1766482332</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>7</v>
+      </c>
+      <c r="B14">
+        <v>95</v>
+      </c>
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="1">
+        <v>301555.15891121957</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>7</v>
+      </c>
+      <c r="B15">
+        <v>50</v>
+      </c>
+      <c r="C15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="1">
+        <v>301873.13141986786</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>7</v>
+      </c>
+      <c r="B16">
+        <v>98</v>
+      </c>
+      <c r="C16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="1">
+        <v>1004256.0955083306</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>7</v>
+      </c>
+      <c r="B17">
+        <v>100</v>
+      </c>
+      <c r="C17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="1">
+        <v>443651.67416058201</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>9</v>
+      </c>
+      <c r="B18">
+        <v>135</v>
+      </c>
+      <c r="C18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" s="1">
+        <v>452752.94221847464</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>9</v>
+      </c>
+      <c r="B19">
         <v>146</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C19" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="1">
-        <v>679666.25696659449</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="D19" s="1">
+        <v>480583.9418052017</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20">
         <v>9</v>
       </c>
-      <c r="B5">
-        <v>142</v>
-      </c>
-      <c r="C5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="1">
-        <v>116765.18564204073</v>
+      <c r="B20">
+        <v>148</v>
+      </c>
+      <c r="C20" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" s="1">
+        <v>481081.15597632382</v>
       </c>
     </row>
   </sheetData>

</xml_diff>